<commit_message>
Balans: hyresrätter förutsägbara, Bostadsveteranen svagare
- Hyresrättsleken: färre plus/minus/direkt, fem 'inget' (105 händelsekort).
- Bostadsveteranen: ingen duellbonus; senior = gratis att röja varningar på hyresrätter.
- Motorn: kalibreringsrattar för att ta bort kort ur lekar och byta yieldspann.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JCFLjpHxkTTwZndbAW5eBH
</commit_message>
<xml_diff>
--- a/kortdata/F_händelsekort.xlsx
+++ b/kortdata/F_händelsekort.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I107"/>
+  <dimension ref="A1:I106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -626,7 +626,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>dolt_plus_dn</t>
+          <t>dolt_minus_dn</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -637,12 +637,12 @@
       <c r="F5" s="2" t="inlineStr"/>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Skötsamma hyresgäster stannar</t>
+          <t>Lägenhet står tom</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>Låg omflyttning ger stabila intäkter och färre inflyttningskostnader.</t>
+          <t>Uppsägning och flyttstädning drar ut på tiden innan ny hyresgäst hittas.</t>
         </is>
       </c>
       <c r="I5" s="2" t="n">
@@ -665,7 +665,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>dolt_plus_dn</t>
+          <t>dolt_minus_dn</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -676,12 +676,12 @@
       <c r="F6" s="2" t="inlineStr"/>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Garageplatser fulltecknade</t>
+          <t>Andrahandsuthyrning upptäcks</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>Alla bilplatser i garaget är uthyrda för första gången på länge.</t>
+          <t>Hyresgästen har hyrt ut svart. Hyresintäkten uteblir under utredningen.</t>
         </is>
       </c>
       <c r="I6" s="2" t="n">
@@ -704,7 +704,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>dolt_plus_dn</t>
+          <t>energi_plus</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
@@ -715,12 +715,12 @@
       <c r="F7" s="2" t="inlineStr"/>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Tvättstugebokningar ökar</t>
+          <t>Nya termostatventiler monteras</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>Fler hyresgäster nyttjar tvättstugan och lägenhetsförrådet mot avgift.</t>
+          <t>Injustering av värmesystemet ger bättre reglering än beräknat.</t>
         </is>
       </c>
       <c r="I7" s="2" t="n">
@@ -743,7 +743,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>dolt_minus_dn</t>
+          <t>energi_minus</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -754,12 +754,12 @@
       <c r="F8" s="2" t="inlineStr"/>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Lägenhet står tom</t>
+          <t>Fjärrvärmeväxlare åldras</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Uppsägning och flyttstädning drar ut på tiden innan ny hyresgäst hittas.</t>
+          <t>Växlaren är original från byggåret och tappar verkningsgrad.</t>
         </is>
       </c>
       <c r="I8" s="2" t="n">
@@ -782,23 +782,27 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>dolt_minus_dn</t>
+          <t>underhallsvarning</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>nej</t>
-        </is>
-      </c>
-      <c r="F9" s="2" t="inlineStr"/>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>Andrahandsuthyrning upptäcks</t>
+          <t>Stammar i akut behov av byte</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>Hyresgästen har hyrt ut svart. Hyresintäkten uteblir under utredningen.</t>
+          <t>Avloppsstammarna är uttjänta och läcker i flera våningsplan.</t>
         </is>
       </c>
       <c r="I9" s="2" t="n">
@@ -821,23 +825,27 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>dolt_minus_dn</t>
+          <t>underhallsvarning</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>nej</t>
-        </is>
-      </c>
-      <c r="F10" s="2" t="inlineStr"/>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Källarförråd vattenskadat</t>
+          <t>Taket läcker vid slagregn</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>Mindre läcka i grunden skadar hyresgästernas förvaring.</t>
+          <t>Papptäckningen har passerat sin livslängd och släpper in vatten.</t>
         </is>
       </c>
       <c r="I10" s="2" t="n">
@@ -860,23 +868,27 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>energi_plus</t>
+          <t>underhallsvarning</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>nej</t>
-        </is>
-      </c>
-      <c r="F11" s="2" t="inlineStr"/>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Nya termostatventiler monteras</t>
+          <t>Hissen klarar inte besiktning</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>Injustering av värmesystemet ger bättre reglering än beräknat.</t>
+          <t>Hissmaskineriet är slitet och måste bytas för att godkännas.</t>
         </is>
       </c>
       <c r="I11" s="2" t="n">
@@ -899,23 +911,23 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>energi_plus</t>
+          <t>villkorskort</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>nej</t>
+          <t>ja</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr"/>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Tätning av fönster lyckas</t>
+          <t>Boverket skärper energikrav</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>Fogar och tätningslister byts i samband med löpande underhåll.</t>
+          <t>Villkor: har fastigheten energiklass D eller sämre blir det −1 DN.</t>
         </is>
       </c>
       <c r="I12" s="2" t="n">
@@ -938,23 +950,23 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>energi_minus</t>
+          <t>villkorskort</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>nej</t>
+          <t>ja</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr"/>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Fjärrvärmeväxlare åldras</t>
+          <t>Portföljen granskas av försäkringsbolag</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>Växlaren är original från byggåret och tappar verkningsgrad.</t>
+          <t>Villkor: äger du 3 eller fler hyresrätter — −1 DN på alla.</t>
         </is>
       </c>
       <c r="I13" s="2" t="n">
@@ -977,7 +989,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>direkt_dn_plus</t>
+          <t>engangskassa_plus</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
@@ -985,15 +997,19 @@
           <t>ja</t>
         </is>
       </c>
-      <c r="F14" s="2" t="inlineStr"/>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Kommunen tecknar blockhyra</t>
+          <t>Retroaktiv hyra betalas ut</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>Kommunen hyr tio lägenheter för nyanlända på ett tioårigt avtal.</t>
+          <t>Hyresnämnden godkänner efterdebiterad hyra för tidigare år.</t>
         </is>
       </c>
       <c r="I14" s="2" t="n">
@@ -1016,7 +1032,7 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>underhallsvarning</t>
+          <t>engangskassa_plus</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
@@ -1026,17 +1042,17 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>Stammar i akut behov av byte</t>
+          <t>Försäkringsersättning för stormskada</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>Avloppsstammarna är uttjänta och läcker i flera våningsplan.</t>
+          <t>Ersättningen täcker mer än den akuta reparationskostnaden.</t>
         </is>
       </c>
       <c r="I15" s="2" t="n">
@@ -1059,7 +1075,7 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>underhallsvarning</t>
+          <t>engangskassa_minus</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
@@ -1074,12 +1090,12 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Taket läcker vid slagregn</t>
+          <t>Akut sanering av mögel</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>Papptäckningen har passerat sin livslängd och släpper in vatten.</t>
+          <t>Fukt bakom kakel har spridit sig och kräver omedelbar åtgärd.</t>
         </is>
       </c>
       <c r="I16" s="2" t="n">
@@ -1102,7 +1118,7 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>underhallsvarning</t>
+          <t>forkop</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
@@ -1110,19 +1126,15 @@
           <t>ja</t>
         </is>
       </c>
-      <c r="F17" s="2" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
+      <c r="F17" s="2" t="inlineStr"/>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>Hissen klarar inte besiktning</t>
+          <t>Tips om hyresfastighet i grannkvarteret</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>Hissmaskineriet är slitet och måste bytas för att godkännas.</t>
+          <t>Behåll på hand. Ger förstaval när en hyresrätt sätts till budgivning.</t>
         </is>
       </c>
       <c r="I17" s="2" t="n">
@@ -1145,7 +1157,7 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>villkorskort</t>
+          <t>forkop</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
@@ -1156,12 +1168,12 @@
       <c r="F18" s="2" t="inlineStr"/>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>Boverket skärper energikrav</t>
+          <t>Mäklarkontakt i bostadsbolaget</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>Villkor: har fastigheten energiklass D eller sämre blir det −1 DN.</t>
+          <t>Behåll på hand. Kortet ger dig förstaval nästa gång en hyresrätt går till budgivning.</t>
         </is>
       </c>
       <c r="I18" s="2" t="n">
@@ -1184,7 +1196,7 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>villkorskort</t>
+          <t>utveckling</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
@@ -1195,12 +1207,12 @@
       <c r="F19" s="2" t="inlineStr"/>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>Portföljen granskas av försäkringsbolag</t>
+          <t>Lyckad hyresförhandling</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>Villkor: äger du 3 eller fler hyresrätter — −1 DN på alla.</t>
+          <t>Förhandlingen med hyresgästföreningen går smidigt och ger erfarenhet. Lägg en utvecklingsbricka på din FC om den har fastighetens typ, annars på din FS.</t>
         </is>
       </c>
       <c r="I19" s="2" t="n">
@@ -1223,7 +1235,7 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>engangskassa_plus</t>
+          <t>riskbuffert</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
@@ -1231,19 +1243,15 @@
           <t>ja</t>
         </is>
       </c>
-      <c r="F20" s="2" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
+      <c r="F20" s="2" t="inlineStr"/>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>Retroaktiv hyra betalas ut</t>
+          <t>Skadefritt år belönas</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>Hyresnämnden godkänner efterdebiterad hyra för tidigare år.</t>
+          <t>Försäkringsbolaget sänker självrisken efter ett år utan skador. Ta en riskbuffert.</t>
         </is>
       </c>
       <c r="I20" s="2" t="n">
@@ -1266,7 +1274,7 @@
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>engangskassa_plus</t>
+          <t>inget</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
@@ -1274,19 +1282,15 @@
           <t>ja</t>
         </is>
       </c>
-      <c r="F21" s="2" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
+      <c r="F21" s="2" t="inlineStr"/>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>Försäkringsersättning för stormskada</t>
+          <t>Lugnt kvartal i huset</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>Ersättningen täcker mer än den akuta reparationskostnaden.</t>
+          <t>Inga felanmälningar utöver det vanliga. Hyrorna kommer in som de ska.</t>
         </is>
       </c>
       <c r="I21" s="2" t="n">
@@ -1309,7 +1313,7 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>engangskassa_minus</t>
+          <t>inget</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
@@ -1317,19 +1321,15 @@
           <t>ja</t>
         </is>
       </c>
-      <c r="F22" s="2" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
+      <c r="F22" s="2" t="inlineStr"/>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>Akut sanering av mögel</t>
+          <t>Hyresavierna går ut som vanligt</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>Fukt bakom kakel har spridit sig och kräver omedelbar åtgärd.</t>
+          <t>Alla betalar i tid. Ingenting att rapportera till styrelsen.</t>
         </is>
       </c>
       <c r="I22" s="2" t="n">
@@ -1352,7 +1352,7 @@
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>forkop</t>
+          <t>inget</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
@@ -1363,12 +1363,12 @@
       <c r="F23" s="2" t="inlineStr"/>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>Tips om hyresfastighet i grannkvarteret</t>
+          <t>Ordinarie fastighetsskötsel</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>Behåll på hand. Ger förstaval när en hyresrätt sätts till budgivning.</t>
+          <t>Gräsklippning, trappstädning och byte av glödlampor. Precis som planerat.</t>
         </is>
       </c>
       <c r="I23" s="2" t="n">
@@ -1391,7 +1391,7 @@
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>forkop</t>
+          <t>inget</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
@@ -1402,12 +1402,12 @@
       <c r="F24" s="2" t="inlineStr"/>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>Mäklarkontakt i bostadsbolaget</t>
+          <t>Årets hyresförhandling klar</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>Behåll på hand. Kortet ger dig förstaval nästa gång en hyresrätt går till budgivning.</t>
+          <t>Hyresgästföreningen och bolaget landar i det väntade. Inga överraskningar.</t>
         </is>
       </c>
       <c r="I24" s="2" t="n">
@@ -1420,33 +1420,33 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>FO-01</t>
+          <t>HR-24</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>FÖRSKOLA</t>
+          <t>HYRESRÄTT</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>dolt_plus_dn</t>
+          <t>inget</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>nej</t>
+          <t>ja</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr"/>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>Kommunen förlänger avtalet</t>
+          <t>Stabilt boende</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>Verksamheten förlänger hyresavtalet med ytterligare fem år.</t>
+          <t>Samma hyresgäster som i fjol. Förutsägbart, tryggt och lite trist.</t>
         </is>
       </c>
       <c r="I25" s="2" t="n">
@@ -1459,7 +1459,7 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>FO-02</t>
+          <t>FO-01</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -1480,12 +1480,12 @@
       <c r="F26" s="2" t="inlineStr"/>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>Fler avdelningar öppnas</t>
+          <t>Kommunen förlänger avtalet</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>Förskolan utökar med en avdelning och hyr angränsande yta.</t>
+          <t>Verksamheten förlänger hyresavtalet med ytterligare fem år.</t>
         </is>
       </c>
       <c r="I26" s="2" t="n">
@@ -1498,7 +1498,7 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>FO-03</t>
+          <t>FO-02</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
@@ -1519,12 +1519,12 @@
       <c r="F27" s="2" t="inlineStr"/>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>Indexklausul ger högre hyra</t>
+          <t>Fler avdelningar öppnas</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>Avtalet räknas upp enligt index utan invändning från kommunen.</t>
+          <t>Förskolan utökar med en avdelning och hyr angränsande yta.</t>
         </is>
       </c>
       <c r="I27" s="2" t="n">
@@ -1537,7 +1537,7 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>FO-04</t>
+          <t>FO-03</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
@@ -1558,12 +1558,12 @@
       <c r="F28" s="2" t="inlineStr"/>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>Föräldrakooperativ flyttar in</t>
+          <t>Indexklausul ger högre hyra</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>Ny huvudman tar över driften och tecknar längre kontrakt.</t>
+          <t>Avtalet räknas upp enligt index utan invändning från kommunen.</t>
         </is>
       </c>
       <c r="I28" s="2" t="n">
@@ -1576,7 +1576,7 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>FO-05</t>
+          <t>FO-04</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
@@ -1597,12 +1597,12 @@
       <c r="F29" s="2" t="inlineStr"/>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>Gården nyttjas av flera verksamheter</t>
+          <t>Föräldrakooperativ flyttar in</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>Kvällsuthyrning av gården till närliggande fritidsgård ger extra intäkt.</t>
+          <t>Ny huvudman tar över driften och tecknar längre kontrakt.</t>
         </is>
       </c>
       <c r="I29" s="2" t="n">
@@ -1615,7 +1615,7 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>FO-06</t>
+          <t>FO-05</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
@@ -1636,12 +1636,12 @@
       <c r="F30" s="2" t="inlineStr"/>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>Köket hyrs ut för catering</t>
+          <t>Gården nyttjas av flera verksamheter</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>Storköket används kvällstid av extern cateringfirma mot avgift.</t>
+          <t>Kvällsuthyrning av gården till närliggande fritidsgård ger extra intäkt.</t>
         </is>
       </c>
       <c r="I30" s="2" t="n">
@@ -1654,7 +1654,7 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>FO-07</t>
+          <t>FO-06</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
@@ -1664,7 +1664,7 @@
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>dolt_minus_dn</t>
+          <t>dolt_plus_dn</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
@@ -1675,12 +1675,12 @@
       <c r="F31" s="2" t="inlineStr"/>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>Avdelning läggs vilande</t>
+          <t>Köket hyrs ut för catering</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>Färre barn i upptagningsområdet gör att en avdelning står tom.</t>
+          <t>Storköket används kvällstid av extern cateringfirma mot avgift.</t>
         </is>
       </c>
       <c r="I31" s="2" t="n">
@@ -1693,7 +1693,7 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>FO-08</t>
+          <t>FO-07</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
@@ -1714,12 +1714,12 @@
       <c r="F32" s="2" t="inlineStr"/>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>Personalutrymme underutnyttjat</t>
+          <t>Avdelning läggs vilande</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>Del av ytan står oanvänd sedan verksamheten omorganiserades.</t>
+          <t>Färre barn i upptagningsområdet gör att en avdelning står tom.</t>
         </is>
       </c>
       <c r="I32" s="2" t="n">
@@ -1732,7 +1732,7 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>FO-09</t>
+          <t>FO-08</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
@@ -1753,12 +1753,12 @@
       <c r="F33" s="2" t="inlineStr"/>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>Fuktskada i grovkök</t>
+          <t>Personalutrymme underutnyttjat</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>Mindre läcka under diskbänken har gått obemärkt förbi ett tag.</t>
+          <t>Del av ytan står oanvänd sedan verksamheten omorganiserades.</t>
         </is>
       </c>
       <c r="I33" s="2" t="n">
@@ -1771,7 +1771,7 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>FO-10</t>
+          <t>FO-09</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
@@ -1781,7 +1781,7 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>energi_plus</t>
+          <t>dolt_minus_dn</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
@@ -1792,12 +1792,12 @@
       <c r="F34" s="2" t="inlineStr"/>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>Solavskärmning minskar kylbehov</t>
+          <t>Fuktskada i grovkök</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>Nya markiser håller nere temperaturen i lekrummen sommartid.</t>
+          <t>Mindre läcka under diskbänken har gått obemärkt förbi ett tag.</t>
         </is>
       </c>
       <c r="I34" s="2" t="n">
@@ -1810,7 +1810,7 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>FO-11</t>
+          <t>FO-10</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
@@ -1831,12 +1831,12 @@
       <c r="F35" s="2" t="inlineStr"/>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>Behovsstyrd ventilation installeras</t>
+          <t>Solavskärmning minskar kylbehov</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>Luftflödet anpassas efter antal barn i lokalen.</t>
+          <t>Nya markiser håller nere temperaturen i lekrummen sommartid.</t>
         </is>
       </c>
       <c r="I35" s="2" t="n">
@@ -1849,7 +1849,7 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>FO-12</t>
+          <t>FO-11</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
@@ -1859,7 +1859,7 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>energi_minus</t>
+          <t>energi_plus</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
@@ -1870,12 +1870,12 @@
       <c r="F36" s="2" t="inlineStr"/>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>Undercentralen är original</t>
+          <t>Behovsstyrd ventilation installeras</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>Värmeväxlaren från byggåret börjar tappa i effektivitet.</t>
+          <t>Luftflödet anpassas efter antal barn i lokalen.</t>
         </is>
       </c>
       <c r="I36" s="2" t="n">
@@ -1888,7 +1888,7 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>FO-13</t>
+          <t>FO-12</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
@@ -1898,23 +1898,23 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>direkt_dn_plus</t>
+          <t>energi_minus</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>nej</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr"/>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>Kommunen bygger ut avtalet till hela huset</t>
+          <t>Undercentralen är original</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>Kommunen tecknar långt hyresavtal för hela fastigheten inklusive tillbyggnad.</t>
+          <t>Värmeväxlaren från byggåret börjar tappa i effektivitet.</t>
         </is>
       </c>
       <c r="I37" s="2" t="n">
@@ -1927,7 +1927,7 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>FO-14</t>
+          <t>FO-13</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -1937,7 +1937,7 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>underhallsvarning</t>
+          <t>direkt_dn_plus</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
@@ -1945,19 +1945,15 @@
           <t>ja</t>
         </is>
       </c>
-      <c r="F38" s="2" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
+      <c r="F38" s="2" t="inlineStr"/>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>Lekutrustningen underkänns</t>
+          <t>Kommunen bygger ut avtalet till hela huset</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>Rutschkana och klätterställning klarar inte säkerhetsbesiktningen.</t>
+          <t>Kommunen tecknar långt hyresavtal för hela fastigheten inklusive tillbyggnad.</t>
         </is>
       </c>
       <c r="I38" s="2" t="n">
@@ -1970,7 +1966,7 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>FO-15</t>
+          <t>FO-14</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
@@ -1990,17 +1986,17 @@
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>Ventilationen klarar inte OVK</t>
+          <t>Lekutrustningen underkänns</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>Luftflödena i lekrummen understiger kraven och kräver ombyggnad.</t>
+          <t>Rutschkana och klätterställning klarar inte säkerhetsbesiktningen.</t>
         </is>
       </c>
       <c r="I39" s="2" t="n">
@@ -2013,7 +2009,7 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>FO-16</t>
+          <t>FO-15</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
@@ -2038,12 +2034,12 @@
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>Fasaden har frostsprängts</t>
+          <t>Ventilationen klarar inte OVK</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>Putsen släpper i stora fält och måste lagas före vintern.</t>
+          <t>Luftflödena i lekrummen understiger kraven och kräver ombyggnad.</t>
         </is>
       </c>
       <c r="I40" s="2" t="n">
@@ -2056,7 +2052,7 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>FO-17</t>
+          <t>FO-16</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
@@ -2066,7 +2062,7 @@
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>villkorskort</t>
+          <t>underhallsvarning</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
@@ -2074,15 +2070,19 @@
           <t>ja</t>
         </is>
       </c>
-      <c r="F41" s="2" t="inlineStr"/>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>Kommunen inför skärpta miljökrav</t>
+          <t>Fasaden har frostsprängts</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>Villkor: ligger energiklassen på D eller sämre dras 1 DN.</t>
+          <t>Putsen släpper i stora fält och måste lagas före vintern.</t>
         </is>
       </c>
       <c r="I41" s="2" t="n">
@@ -2095,7 +2095,7 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>FO-18</t>
+          <t>FO-17</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
@@ -2116,12 +2116,12 @@
       <c r="F42" s="2" t="inlineStr"/>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>Skolinspektionen granskar fastighetsbeståndet</t>
+          <t>Kommunen inför skärpta miljökrav</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>Villkor: äger du 3 eller fler förskolor — −1 DN på alla.</t>
+          <t>Villkor: ligger energiklassen på D eller sämre dras 1 DN.</t>
         </is>
       </c>
       <c r="I42" s="2" t="n">
@@ -2134,7 +2134,7 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>FO-19</t>
+          <t>FO-18</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
@@ -2144,7 +2144,7 @@
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>engangskassa_plus</t>
+          <t>villkorskort</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
@@ -2152,19 +2152,15 @@
           <t>ja</t>
         </is>
       </c>
-      <c r="F43" s="2" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
+      <c r="F43" s="2" t="inlineStr"/>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>Kommunalt underhållsbidrag betalas ut</t>
+          <t>Skolinspektionen granskar fastighetsbeståndet</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>Bidraget täcker mer än den planerade underhållsåtgärden.</t>
+          <t>Villkor: äger du 3 eller fler förskolor — −1 DN på alla.</t>
         </is>
       </c>
       <c r="I43" s="2" t="n">
@@ -2177,7 +2173,7 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>FO-20</t>
+          <t>FO-19</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
@@ -2197,17 +2193,17 @@
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>Försäkringsersättning för skadegörelse</t>
+          <t>Kommunalt underhållsbidrag betalas ut</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>Ersättningen från inbrottet överstiger reparationskostnaden.</t>
+          <t>Bidraget täcker mer än den planerade underhållsåtgärden.</t>
         </is>
       </c>
       <c r="I44" s="2" t="n">
@@ -2220,7 +2216,7 @@
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>FO-21</t>
+          <t>FO-20</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
@@ -2240,17 +2236,17 @@
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>Statligt investeringsstöd för förskolor</t>
+          <t>Försäkringsersättning för skadegörelse</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>Fastigheten kvalificerar för stöd till förbättrad barnmiljö.</t>
+          <t>Ersättningen från inbrottet överstiger reparationskostnaden.</t>
         </is>
       </c>
       <c r="I45" s="2" t="n">
@@ -2263,7 +2259,7 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>FO-22</t>
+          <t>FO-21</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
@@ -2273,7 +2269,7 @@
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>forkop</t>
+          <t>engangskassa_plus</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
@@ -2281,15 +2277,19 @@
           <t>ja</t>
         </is>
       </c>
-      <c r="F46" s="2" t="inlineStr"/>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>Tips om förskola på kommunens lista</t>
+          <t>Statligt investeringsstöd för förskolor</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>Behåll på hand. Ger förstaval när en förskola sätts till budgivning.</t>
+          <t>Fastigheten kvalificerar för stöd till förbättrad barnmiljö.</t>
         </is>
       </c>
       <c r="I46" s="2" t="n">
@@ -2302,7 +2302,7 @@
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>FO-23</t>
+          <t>FO-22</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
@@ -2323,12 +2323,12 @@
       <c r="F47" s="2" t="inlineStr"/>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>Kontakt på kommunens fastighetskontor</t>
+          <t>Tips om förskola på kommunens lista</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t>Behåll på hand. Kortet ger dig förstaval nästa gång en förskola går till budgivning.</t>
+          <t>Behåll på hand. Ger förstaval när en förskola sätts till budgivning.</t>
         </is>
       </c>
       <c r="I47" s="2" t="n">
@@ -2341,33 +2341,33 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>LO-01</t>
+          <t>FO-23</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>LOKAL</t>
+          <t>FÖRSKOLA</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>dolt_plus_dn</t>
+          <t>forkop</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>nej</t>
+          <t>ja</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr"/>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>Omsättningshyra slår väl ut</t>
+          <t>Kontakt på kommunens fastighetskontor</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
-          <t>Butikens julförsäljning ger högre omsättningshyra än väntat.</t>
+          <t>Behåll på hand. Kortet ger dig förstaval nästa gång en förskola går till budgivning.</t>
         </is>
       </c>
       <c r="I48" s="2" t="n">
@@ -2380,7 +2380,7 @@
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>LO-02</t>
+          <t>LO-01</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
@@ -2401,12 +2401,12 @@
       <c r="F49" s="2" t="inlineStr"/>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>Ny hyresgäst tecknar långt kontrakt</t>
+          <t>Omsättningshyra slår väl ut</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
-          <t>Kedjebutik flyttar in på ett femårsavtal med indexklausul.</t>
+          <t>Butikens julförsäljning ger högre omsättningshyra än väntat.</t>
         </is>
       </c>
       <c r="I49" s="2" t="n">
@@ -2419,7 +2419,7 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>LO-03</t>
+          <t>LO-02</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
@@ -2440,12 +2440,12 @@
       <c r="F50" s="2" t="inlineStr"/>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>Skyltläget lockar ny verksamhet</t>
+          <t>Ny hyresgäst tecknar långt kontrakt</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
-          <t>Ett gynnsamt gathörn gör att hyresgästen kan ta ut högre hyra.</t>
+          <t>Kedjebutik flyttar in på ett femårsavtal med indexklausul.</t>
         </is>
       </c>
       <c r="I50" s="2" t="n">
@@ -2458,7 +2458,7 @@
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>LO-04</t>
+          <t>LO-03</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
@@ -2479,12 +2479,12 @@
       <c r="F51" s="2" t="inlineStr"/>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>Restaurangen bygger ut uteserveringen</t>
+          <t>Skyltläget lockar ny verksamhet</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr">
         <is>
-          <t>Utökad serveringsyta höjer hyresintäkten under sommarhalvåret.</t>
+          <t>Ett gynnsamt gathörn gör att hyresgästen kan ta ut högre hyra.</t>
         </is>
       </c>
       <c r="I51" s="2" t="n">
@@ -2497,7 +2497,7 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>LO-05</t>
+          <t>LO-04</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
@@ -2518,12 +2518,12 @@
       <c r="F52" s="2" t="inlineStr"/>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>Popup-butik hyr in sig kort</t>
+          <t>Restaurangen bygger ut uteserveringen</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr">
         <is>
-          <t>Ledig lokal fylls tillfälligt av kampanjhyresgäst mellan avtal.</t>
+          <t>Utökad serveringsyta höjer hyresintäkten under sommarhalvåret.</t>
         </is>
       </c>
       <c r="I52" s="2" t="n">
@@ -2536,7 +2536,7 @@
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>LO-06</t>
+          <t>LO-05</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
@@ -2546,7 +2546,7 @@
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>dolt_minus_dn</t>
+          <t>dolt_plus_dn</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
@@ -2557,12 +2557,12 @@
       <c r="F53" s="2" t="inlineStr"/>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>Butiken sänker sin omsättning</t>
+          <t>Popup-butik hyr in sig kort</t>
         </is>
       </c>
       <c r="H53" s="2" t="inlineStr">
         <is>
-          <t>Minskad handel gör att omsättningshyran blir lägre än budgeterat.</t>
+          <t>Ledig lokal fylls tillfälligt av kampanjhyresgäst mellan avtal.</t>
         </is>
       </c>
       <c r="I53" s="2" t="n">
@@ -2575,7 +2575,7 @@
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>LO-07</t>
+          <t>LO-06</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
@@ -2596,12 +2596,12 @@
       <c r="F54" s="2" t="inlineStr"/>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>Lokal svår att hyra ut vidare</t>
+          <t>Butiken sänker sin omsättning</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr">
         <is>
-          <t>Ovanlig planlösning gör att uthyrningen drar ut på tiden.</t>
+          <t>Minskad handel gör att omsättningshyran blir lägre än budgeterat.</t>
         </is>
       </c>
       <c r="I54" s="2" t="n">
@@ -2614,7 +2614,7 @@
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>LO-08</t>
+          <t>LO-07</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
@@ -2635,12 +2635,12 @@
       <c r="F55" s="2" t="inlineStr"/>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>Konkurrerande handelsplats öppnar</t>
+          <t>Lokal svår att hyra ut vidare</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr">
         <is>
-          <t>Kunderna söker sig till nytt köpcentrum i närheten.</t>
+          <t>Ovanlig planlösning gör att uthyrningen drar ut på tiden.</t>
         </is>
       </c>
       <c r="I55" s="2" t="n">
@@ -2653,7 +2653,7 @@
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>LO-09</t>
+          <t>LO-08</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
@@ -2674,12 +2674,12 @@
       <c r="F56" s="2" t="inlineStr"/>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>Fettavskiljaren läcker smått</t>
+          <t>Konkurrerande handelsplats öppnar</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
         <is>
-          <t>Mindre läckage i restauranglokalens avlopp har gått obemärkt förbi.</t>
+          <t>Kunderna söker sig till nytt köpcentrum i närheten.</t>
         </is>
       </c>
       <c r="I56" s="2" t="n">
@@ -2692,7 +2692,7 @@
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>LO-10</t>
+          <t>LO-09</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
@@ -2713,12 +2713,12 @@
       <c r="F57" s="2" t="inlineStr"/>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>Skyltfönster krossat en tid</t>
+          <t>Fettavskiljaren läcker smått</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
         <is>
-          <t>Reparation dröjer och lokalen syns sämre mot gatan.</t>
+          <t>Mindre läckage i restauranglokalens avlopp har gått obemärkt förbi.</t>
         </is>
       </c>
       <c r="I57" s="2" t="n">
@@ -2731,7 +2731,7 @@
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>LO-11</t>
+          <t>LO-10</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
@@ -2752,12 +2752,12 @@
       <c r="F58" s="2" t="inlineStr"/>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>Hyresrabatt förhandlas fram i det tysta</t>
+          <t>Skyltfönster krossat en tid</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr">
         <is>
-          <t>Hyresgästen får tillfällig rabatt för att inte flytta.</t>
+          <t>Reparation dröjer och lokalen syns sämre mot gatan.</t>
         </is>
       </c>
       <c r="I58" s="2" t="n">
@@ -2770,7 +2770,7 @@
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>LO-12</t>
+          <t>LO-11</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
@@ -2780,7 +2780,7 @@
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>energi_plus</t>
+          <t>dolt_minus_dn</t>
         </is>
       </c>
       <c r="E59" s="2" t="inlineStr">
@@ -2791,12 +2791,12 @@
       <c r="F59" s="2" t="inlineStr"/>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>Ny LED-belysning i butiksytan</t>
+          <t>Hyresrabatt förhandlas fram i det tysta</t>
         </is>
       </c>
       <c r="H59" s="2" t="inlineStr">
         <is>
-          <t>Hyresgästen byter armaturer och sänker fastighetens elkostnad.</t>
+          <t>Hyresgästen får tillfällig rabatt för att inte flytta.</t>
         </is>
       </c>
       <c r="I59" s="2" t="n">
@@ -2809,7 +2809,7 @@
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>LO-13</t>
+          <t>LO-12</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
@@ -2819,7 +2819,7 @@
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>energi_minus</t>
+          <t>energi_plus</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
@@ -2830,12 +2830,12 @@
       <c r="F60" s="2" t="inlineStr"/>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t>Kylanläggningen börjar dra mer el</t>
+          <t>Ny LED-belysning i butiksytan</t>
         </is>
       </c>
       <c r="H60" s="2" t="inlineStr">
         <is>
-          <t>Kompressorn i livsmedelsbutikens kyla närmar sig sin livslängd.</t>
+          <t>Hyresgästen byter armaturer och sänker fastighetens elkostnad.</t>
         </is>
       </c>
       <c r="I60" s="2" t="n">
@@ -2848,7 +2848,7 @@
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>LO-14</t>
+          <t>LO-13</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
@@ -2869,12 +2869,12 @@
       <c r="F61" s="2" t="inlineStr"/>
       <c r="G61" s="2" t="inlineStr">
         <is>
-          <t>Ventilationsaggregatet är original</t>
+          <t>Kylanläggningen börjar dra mer el</t>
         </is>
       </c>
       <c r="H61" s="2" t="inlineStr">
         <is>
-          <t>Aggregatet från byggåret har sämre verkningsgrad än moderna system.</t>
+          <t>Kompressorn i livsmedelsbutikens kyla närmar sig sin livslängd.</t>
         </is>
       </c>
       <c r="I61" s="2" t="n">
@@ -2887,7 +2887,7 @@
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>LO-15</t>
+          <t>LO-14</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
@@ -2897,23 +2897,23 @@
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>direkt_dn_plus</t>
+          <t>energi_minus</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>nej</t>
         </is>
       </c>
       <c r="F62" s="2" t="inlineStr"/>
       <c r="G62" s="2" t="inlineStr">
         <is>
-          <t>Ankarhyresgäst tecknar tioårsavtal</t>
+          <t>Ventilationsaggregatet är original</t>
         </is>
       </c>
       <c r="H62" s="2" t="inlineStr">
         <is>
-          <t>Stor kedjebutik flyttar in och lyfter hela husets attraktionskraft.</t>
+          <t>Aggregatet från byggåret har sämre verkningsgrad än moderna system.</t>
         </is>
       </c>
       <c r="I62" s="2" t="n">
@@ -2926,7 +2926,7 @@
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>LO-16</t>
+          <t>LO-15</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
@@ -2936,7 +2936,7 @@
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>direkt_dn_minus</t>
+          <t>direkt_dn_plus</t>
         </is>
       </c>
       <c r="E63" s="2" t="inlineStr">
@@ -2947,12 +2947,12 @@
       <c r="F63" s="2" t="inlineStr"/>
       <c r="G63" s="2" t="inlineStr">
         <is>
-          <t>Ankarhyresgästen går i konkurs</t>
+          <t>Ankarhyresgäst tecknar tioårsavtal</t>
         </is>
       </c>
       <c r="H63" s="2" t="inlineStr">
         <is>
-          <t>Den stora hyresgästen lämnar utan uppsägningstid och lokalen står tom.</t>
+          <t>Stor kedjebutik flyttar in och lyfter hela husets attraktionskraft.</t>
         </is>
       </c>
       <c r="I63" s="2" t="n">
@@ -2965,7 +2965,7 @@
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>LO-17</t>
+          <t>LO-16</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
@@ -2975,7 +2975,7 @@
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>underhallsvarning</t>
+          <t>direkt_dn_minus</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
@@ -2983,19 +2983,15 @@
           <t>ja</t>
         </is>
       </c>
-      <c r="F64" s="2" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
+      <c r="F64" s="2" t="inlineStr"/>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>Golvet i handelslokalen är utslitet</t>
+          <t>Ankarhyresgästen går i konkurs</t>
         </is>
       </c>
       <c r="H64" s="2" t="inlineStr">
         <is>
-          <t>Betonggolvet måste slipas och beläggas på nytt.</t>
+          <t>Den stora hyresgästen lämnar utan uppsägningstid och lokalen står tom.</t>
         </is>
       </c>
       <c r="I64" s="2" t="n">
@@ -3008,7 +3004,7 @@
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>LO-18</t>
+          <t>LO-17</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
@@ -3028,17 +3024,17 @@
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr">
         <is>
-          <t>Fasaden mot gatan vittrar</t>
+          <t>Golvet i handelslokalen är utslitet</t>
         </is>
       </c>
       <c r="H65" s="2" t="inlineStr">
         <is>
-          <t>Putsskador och lossnande fasadplattor måste åtgärdas.</t>
+          <t>Betonggolvet måste slipas och beläggas på nytt.</t>
         </is>
       </c>
       <c r="I65" s="2" t="n">
@@ -3051,7 +3047,7 @@
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>LO-19</t>
+          <t>LO-18</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
@@ -3061,7 +3057,7 @@
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>villkorskort</t>
+          <t>underhallsvarning</t>
         </is>
       </c>
       <c r="E66" s="2" t="inlineStr">
@@ -3069,15 +3065,19 @@
           <t>ja</t>
         </is>
       </c>
-      <c r="F66" s="2" t="inlineStr"/>
+      <c r="F66" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>E-handeln tar ytterligare mark</t>
+          <t>Fasaden mot gatan vittrar</t>
         </is>
       </c>
       <c r="H66" s="2" t="inlineStr">
         <is>
-          <t>Villkor: äger du 3 eller fler lokaler — −1 DN på alla.</t>
+          <t>Putsskador och lossnande fasadplattor måste åtgärdas.</t>
         </is>
       </c>
       <c r="I66" s="2" t="n">
@@ -3090,7 +3090,7 @@
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>LO-20</t>
+          <t>LO-19</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
@@ -3111,12 +3111,12 @@
       <c r="F67" s="2" t="inlineStr"/>
       <c r="G67" s="2" t="inlineStr">
         <is>
-          <t>Kommunen skärper energikrav för handel</t>
+          <t>E-handeln tar ytterligare mark</t>
         </is>
       </c>
       <c r="H67" s="2" t="inlineStr">
         <is>
-          <t>Villkor: energiklass D eller sämre ger −1 DN på fastigheten.</t>
+          <t>Villkor: äger du 3 eller fler lokaler — −1 DN på alla.</t>
         </is>
       </c>
       <c r="I67" s="2" t="n">
@@ -3129,7 +3129,7 @@
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>LO-21</t>
+          <t>LO-20</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
@@ -3139,7 +3139,7 @@
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>engangskassa_plus</t>
+          <t>villkorskort</t>
         </is>
       </c>
       <c r="E68" s="2" t="inlineStr">
@@ -3147,19 +3147,15 @@
           <t>ja</t>
         </is>
       </c>
-      <c r="F68" s="2" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
+      <c r="F68" s="2" t="inlineStr"/>
       <c r="G68" s="2" t="inlineStr">
         <is>
-          <t>Avflyttande hyresgäst betalar avgångsvederlag</t>
+          <t>Kommunen skärper energikrav för handel</t>
         </is>
       </c>
       <c r="H68" s="2" t="inlineStr">
         <is>
-          <t>Hyresgästen löser ut sig ur kontraktet i förtid.</t>
+          <t>Villkor: energiklass D eller sämre ger −1 DN på fastigheten.</t>
         </is>
       </c>
       <c r="I68" s="2" t="n">
@@ -3172,7 +3168,7 @@
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>LO-22</t>
+          <t>LO-21</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr">
@@ -3192,17 +3188,17 @@
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
         <is>
-          <t>Försäkringsersättning efter vattenskada</t>
+          <t>Avflyttande hyresgäst betalar avgångsvederlag</t>
         </is>
       </c>
       <c r="H69" s="2" t="inlineStr">
         <is>
-          <t>Ersättningen från skyfallet täcker mer än saneringskostnaden.</t>
+          <t>Hyresgästen löser ut sig ur kontraktet i förtid.</t>
         </is>
       </c>
       <c r="I69" s="2" t="n">
@@ -3215,7 +3211,7 @@
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>LO-23</t>
+          <t>LO-22</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
@@ -3225,7 +3221,7 @@
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>engangskassa_minus</t>
+          <t>engangskassa_plus</t>
         </is>
       </c>
       <c r="E70" s="2" t="inlineStr">
@@ -3235,17 +3231,17 @@
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G70" s="2" t="inlineStr">
         <is>
-          <t>Akutsanering av fettavskiljare</t>
+          <t>Försäkringsersättning efter vattenskada</t>
         </is>
       </c>
       <c r="H70" s="2" t="inlineStr">
         <is>
-          <t>Avskiljaren är överfull och måste tömmas och åtgärdas omgående.</t>
+          <t>Ersättningen från skyfallet täcker mer än saneringskostnaden.</t>
         </is>
       </c>
       <c r="I70" s="2" t="n">
@@ -3258,7 +3254,7 @@
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>LO-24</t>
+          <t>LO-23</t>
         </is>
       </c>
       <c r="C71" s="2" t="inlineStr">
@@ -3278,17 +3274,17 @@
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G71" s="2" t="inlineStr">
         <is>
-          <t>Klotter saneras akut på fasaden</t>
+          <t>Akutsanering av fettavskiljare</t>
         </is>
       </c>
       <c r="H71" s="2" t="inlineStr">
         <is>
-          <t>Fasaden klottras ned upprepade gånger och kräver skyddsbehandling.</t>
+          <t>Avskiljaren är överfull och måste tömmas och åtgärdas omgående.</t>
         </is>
       </c>
       <c r="I71" s="2" t="n">
@@ -3301,7 +3297,7 @@
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>LO-25</t>
+          <t>LO-24</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
@@ -3311,7 +3307,7 @@
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>forkop</t>
+          <t>engangskassa_minus</t>
         </is>
       </c>
       <c r="E72" s="2" t="inlineStr">
@@ -3319,15 +3315,19 @@
           <t>ja</t>
         </is>
       </c>
-      <c r="F72" s="2" t="inlineStr"/>
+      <c r="F72" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
       <c r="G72" s="2" t="inlineStr">
         <is>
-          <t>Tips om butikslokal i köpstark gata</t>
+          <t>Klotter saneras akut på fasaden</t>
         </is>
       </c>
       <c r="H72" s="2" t="inlineStr">
         <is>
-          <t>Behåll på hand. Ger förstaval när en lokal sätts till budgivning.</t>
+          <t>Fasaden klottras ned upprepade gånger och kräver skyddsbehandling.</t>
         </is>
       </c>
       <c r="I72" s="2" t="n">
@@ -3340,7 +3340,7 @@
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>LO-26</t>
+          <t>LO-25</t>
         </is>
       </c>
       <c r="C73" s="2" t="inlineStr">
@@ -3361,12 +3361,12 @@
       <c r="F73" s="2" t="inlineStr"/>
       <c r="G73" s="2" t="inlineStr">
         <is>
-          <t>Kontakt hos fastighetsmäklare i city</t>
+          <t>Tips om butikslokal i köpstark gata</t>
         </is>
       </c>
       <c r="H73" s="2" t="inlineStr">
         <is>
-          <t>Behåll på hand. Kortet ger dig förstaval nästa gång en lokal går till budgivning.</t>
+          <t>Behåll på hand. Ger förstaval när en lokal sätts till budgivning.</t>
         </is>
       </c>
       <c r="I73" s="2" t="n">
@@ -3379,33 +3379,33 @@
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>KO-01</t>
+          <t>LO-26</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>KONTOR</t>
+          <t>LOKAL</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>dolt_plus_dn</t>
+          <t>forkop</t>
         </is>
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>nej</t>
+          <t>ja</t>
         </is>
       </c>
       <c r="F74" s="2" t="inlineStr"/>
       <c r="G74" s="2" t="inlineStr">
         <is>
-          <t>Hyresgästen expanderar på plats</t>
+          <t>Kontakt hos fastighetsmäklare i city</t>
         </is>
       </c>
       <c r="H74" s="2" t="inlineStr">
         <is>
-          <t>Företaget hyr angränsande yta i samband med tillväxt.</t>
+          <t>Behåll på hand. Kortet ger dig förstaval nästa gång en lokal går till budgivning.</t>
         </is>
       </c>
       <c r="I74" s="2" t="n">
@@ -3418,7 +3418,7 @@
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>KO-02</t>
+          <t>KO-01</t>
         </is>
       </c>
       <c r="C75" s="2" t="inlineStr">
@@ -3439,12 +3439,12 @@
       <c r="F75" s="2" t="inlineStr"/>
       <c r="G75" s="2" t="inlineStr">
         <is>
-          <t>Långt avtal förlängs i förtid</t>
+          <t>Hyresgästen expanderar på plats</t>
         </is>
       </c>
       <c r="H75" s="2" t="inlineStr">
         <is>
-          <t>Hyresgästen tecknar nytt avtal två år innan det gamla löper ut.</t>
+          <t>Företaget hyr angränsande yta i samband med tillväxt.</t>
         </is>
       </c>
       <c r="I75" s="2" t="n">
@@ -3457,7 +3457,7 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>KO-03</t>
+          <t>KO-02</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
@@ -3478,12 +3478,12 @@
       <c r="F76" s="2" t="inlineStr"/>
       <c r="G76" s="2" t="inlineStr">
         <is>
-          <t>Kontorshotell fyller vakanta ytor</t>
+          <t>Långt avtal förlängs i förtid</t>
         </is>
       </c>
       <c r="H76" s="2" t="inlineStr">
         <is>
-          <t>Flexibla korttidskontrakt gör att tomma ytor snabbt hyrs ut.</t>
+          <t>Hyresgästen tecknar nytt avtal två år innan det gamla löper ut.</t>
         </is>
       </c>
       <c r="I76" s="2" t="n">
@@ -3496,7 +3496,7 @@
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>KO-04</t>
+          <t>KO-03</t>
         </is>
       </c>
       <c r="C77" s="2" t="inlineStr">
@@ -3517,12 +3517,12 @@
       <c r="F77" s="2" t="inlineStr"/>
       <c r="G77" s="2" t="inlineStr">
         <is>
-          <t>Indexuppräkning ger högre hyra</t>
+          <t>Kontorshotell fyller vakanta ytor</t>
         </is>
       </c>
       <c r="H77" s="2" t="inlineStr">
         <is>
-          <t>Avtalet räknas upp enligt konsumentprisindex utan omförhandling.</t>
+          <t>Flexibla korttidskontrakt gör att tomma ytor snabbt hyrs ut.</t>
         </is>
       </c>
       <c r="I77" s="2" t="n">
@@ -3535,7 +3535,7 @@
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>KO-05</t>
+          <t>KO-04</t>
         </is>
       </c>
       <c r="C78" s="2" t="inlineStr">
@@ -3545,7 +3545,7 @@
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>dolt_minus_dn</t>
+          <t>dolt_plus_dn</t>
         </is>
       </c>
       <c r="E78" s="2" t="inlineStr">
@@ -3556,12 +3556,12 @@
       <c r="F78" s="2" t="inlineStr"/>
       <c r="G78" s="2" t="inlineStr">
         <is>
-          <t>Del av våningsplan står tomt</t>
+          <t>Indexuppräkning ger högre hyra</t>
         </is>
       </c>
       <c r="H78" s="2" t="inlineStr">
         <is>
-          <t>Hyresgästen har krympt sin yta men avtalet omförhandlas inte förrän nästa period.</t>
+          <t>Avtalet räknas upp enligt konsumentprisindex utan omförhandling.</t>
         </is>
       </c>
       <c r="I78" s="2" t="n">
@@ -3574,7 +3574,7 @@
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>KO-06</t>
+          <t>KO-05</t>
         </is>
       </c>
       <c r="C79" s="2" t="inlineStr">
@@ -3595,12 +3595,12 @@
       <c r="F79" s="2" t="inlineStr"/>
       <c r="G79" s="2" t="inlineStr">
         <is>
-          <t>Distansarbete minskar ytbehovet</t>
+          <t>Del av våningsplan står tomt</t>
         </is>
       </c>
       <c r="H79" s="2" t="inlineStr">
         <is>
-          <t>Hyresgästen nyttjar bara halva sin kontrakterade yta.</t>
+          <t>Hyresgästen har krympt sin yta men avtalet omförhandlas inte förrän nästa period.</t>
         </is>
       </c>
       <c r="I79" s="2" t="n">
@@ -3613,7 +3613,7 @@
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>KO-07</t>
+          <t>KO-06</t>
         </is>
       </c>
       <c r="C80" s="2" t="inlineStr">
@@ -3634,12 +3634,12 @@
       <c r="F80" s="2" t="inlineStr"/>
       <c r="G80" s="2" t="inlineStr">
         <is>
-          <t>Konferensrum står obokat</t>
+          <t>Distansarbete minskar ytbehovet</t>
         </is>
       </c>
       <c r="H80" s="2" t="inlineStr">
         <is>
-          <t>Gemensamma ytor genererar mindre avgiftsintäkt än beräknat.</t>
+          <t>Hyresgästen nyttjar bara halva sin kontrakterade yta.</t>
         </is>
       </c>
       <c r="I80" s="2" t="n">
@@ -3652,7 +3652,7 @@
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>KO-08</t>
+          <t>KO-07</t>
         </is>
       </c>
       <c r="C81" s="2" t="inlineStr">
@@ -3673,12 +3673,12 @@
       <c r="F81" s="2" t="inlineStr"/>
       <c r="G81" s="2" t="inlineStr">
         <is>
-          <t>Elkapaciteten börjar bli en flaskhals</t>
+          <t>Konferensrum står obokat</t>
         </is>
       </c>
       <c r="H81" s="2" t="inlineStr">
         <is>
-          <t>Ökad serverdrift hos hyresgästen belastar fastighetens elnät i det tysta.</t>
+          <t>Gemensamma ytor genererar mindre avgiftsintäkt än beräknat.</t>
         </is>
       </c>
       <c r="I81" s="2" t="n">
@@ -3691,7 +3691,7 @@
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>KO-09</t>
+          <t>KO-08</t>
         </is>
       </c>
       <c r="C82" s="2" t="inlineStr">
@@ -3712,12 +3712,12 @@
       <c r="F82" s="2" t="inlineStr"/>
       <c r="G82" s="2" t="inlineStr">
         <is>
-          <t>Reception underutnyttjad</t>
+          <t>Elkapaciteten börjar bli en flaskhals</t>
         </is>
       </c>
       <c r="H82" s="2" t="inlineStr">
         <is>
-          <t>Delad servicefunktion i entrén ger lägre intäkt än planerat.</t>
+          <t>Ökad serverdrift hos hyresgästen belastar fastighetens elnät i det tysta.</t>
         </is>
       </c>
       <c r="I82" s="2" t="n">
@@ -3730,7 +3730,7 @@
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>KO-10</t>
+          <t>KO-09</t>
         </is>
       </c>
       <c r="C83" s="2" t="inlineStr">
@@ -3751,12 +3751,12 @@
       <c r="F83" s="2" t="inlineStr"/>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>Parkeringsgaraget har lediga platser</t>
+          <t>Reception underutnyttjad</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
         <is>
-          <t>Färre anställda på plats gör att garageintäkterna sjunker.</t>
+          <t>Delad servicefunktion i entrén ger lägre intäkt än planerat.</t>
         </is>
       </c>
       <c r="I83" s="2" t="n">
@@ -3769,7 +3769,7 @@
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>KO-11</t>
+          <t>KO-10</t>
         </is>
       </c>
       <c r="C84" s="2" t="inlineStr">
@@ -3779,7 +3779,7 @@
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>energi_plus</t>
+          <t>dolt_minus_dn</t>
         </is>
       </c>
       <c r="E84" s="2" t="inlineStr">
@@ -3790,12 +3790,12 @@
       <c r="F84" s="2" t="inlineStr"/>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>Behovsstyrd belysning installeras</t>
+          <t>Parkeringsgaraget har lediga platser</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
         <is>
-          <t>Närvarostyrda armaturer sänker elförbrukningen i kontorskorridorerna.</t>
+          <t>Färre anställda på plats gör att garageintäkterna sjunker.</t>
         </is>
       </c>
       <c r="I84" s="2" t="n">
@@ -3808,7 +3808,7 @@
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>KO-12</t>
+          <t>KO-11</t>
         </is>
       </c>
       <c r="C85" s="2" t="inlineStr">
@@ -3818,7 +3818,7 @@
       </c>
       <c r="D85" s="2" t="inlineStr">
         <is>
-          <t>energi_minus</t>
+          <t>energi_plus</t>
         </is>
       </c>
       <c r="E85" s="2" t="inlineStr">
@@ -3829,12 +3829,12 @@
       <c r="F85" s="2" t="inlineStr"/>
       <c r="G85" s="2" t="inlineStr">
         <is>
-          <t>Kylmaskinen för komfortkyla åldras</t>
+          <t>Behovsstyrd belysning installeras</t>
         </is>
       </c>
       <c r="H85" s="2" t="inlineStr">
         <is>
-          <t>Kompressorn börjar dra mer el än när den var ny.</t>
+          <t>Närvarostyrda armaturer sänker elförbrukningen i kontorskorridorerna.</t>
         </is>
       </c>
       <c r="I85" s="2" t="n">
@@ -3847,7 +3847,7 @@
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>KO-13</t>
+          <t>KO-12</t>
         </is>
       </c>
       <c r="C86" s="2" t="inlineStr">
@@ -3868,12 +3868,12 @@
       <c r="F86" s="2" t="inlineStr"/>
       <c r="G86" s="2" t="inlineStr">
         <is>
-          <t>Klimatskalet läcker värme</t>
+          <t>Kylmaskinen för komfortkyla åldras</t>
         </is>
       </c>
       <c r="H86" s="2" t="inlineStr">
         <is>
-          <t>Fönsterpartierna från byggåret har sämre isolerförmåga än moderna glas.</t>
+          <t>Kompressorn börjar dra mer el än när den var ny.</t>
         </is>
       </c>
       <c r="I86" s="2" t="n">
@@ -3886,7 +3886,7 @@
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>KO-14</t>
+          <t>KO-13</t>
         </is>
       </c>
       <c r="C87" s="2" t="inlineStr">
@@ -3896,23 +3896,23 @@
       </c>
       <c r="D87" s="2" t="inlineStr">
         <is>
-          <t>direkt_dn_plus</t>
+          <t>energi_minus</t>
         </is>
       </c>
       <c r="E87" s="2" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>nej</t>
         </is>
       </c>
       <c r="F87" s="2" t="inlineStr"/>
       <c r="G87" s="2" t="inlineStr">
         <is>
-          <t>Storbolag flyttar in på tioårsavtal</t>
+          <t>Klimatskalet läcker värme</t>
         </is>
       </c>
       <c r="H87" s="2" t="inlineStr">
         <is>
-          <t>Ett väletablerat företag hyr hela plan för sitt regionkontor.</t>
+          <t>Fönsterpartierna från byggåret har sämre isolerförmåga än moderna glas.</t>
         </is>
       </c>
       <c r="I87" s="2" t="n">
@@ -3925,7 +3925,7 @@
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>KO-15</t>
+          <t>KO-14</t>
         </is>
       </c>
       <c r="C88" s="2" t="inlineStr">
@@ -3935,7 +3935,7 @@
       </c>
       <c r="D88" s="2" t="inlineStr">
         <is>
-          <t>direkt_dn_minus</t>
+          <t>direkt_dn_plus</t>
         </is>
       </c>
       <c r="E88" s="2" t="inlineStr">
@@ -3946,12 +3946,12 @@
       <c r="F88" s="2" t="inlineStr"/>
       <c r="G88" s="2" t="inlineStr">
         <is>
-          <t>Storhyresgästen flyttar till nybygge</t>
+          <t>Storbolag flyttar in på tioårsavtal</t>
         </is>
       </c>
       <c r="H88" s="2" t="inlineStr">
         <is>
-          <t>Ankarhyresgästen lämnar för modernare lokaler i nybyggt kvarter.</t>
+          <t>Ett väletablerat företag hyr hela plan för sitt regionkontor.</t>
         </is>
       </c>
       <c r="I88" s="2" t="n">
@@ -3964,7 +3964,7 @@
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>KO-16</t>
+          <t>KO-15</t>
         </is>
       </c>
       <c r="C89" s="2" t="inlineStr">
@@ -3985,12 +3985,12 @@
       <c r="F89" s="2" t="inlineStr"/>
       <c r="G89" s="2" t="inlineStr">
         <is>
-          <t>Hyresgästen läggs ner i omorganisation</t>
+          <t>Storhyresgästen flyttar till nybygge</t>
         </is>
       </c>
       <c r="H89" s="2" t="inlineStr">
         <is>
-          <t>Moderbolaget stänger den lokala verksamheten och avtalet upphör.</t>
+          <t>Ankarhyresgästen lämnar för modernare lokaler i nybyggt kvarter.</t>
         </is>
       </c>
       <c r="I89" s="2" t="n">
@@ -4003,7 +4003,7 @@
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>KO-17</t>
+          <t>KO-16</t>
         </is>
       </c>
       <c r="C90" s="2" t="inlineStr">
@@ -4013,7 +4013,7 @@
       </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t>underhallsvarning</t>
+          <t>direkt_dn_minus</t>
         </is>
       </c>
       <c r="E90" s="2" t="inlineStr">
@@ -4021,19 +4021,15 @@
           <t>ja</t>
         </is>
       </c>
-      <c r="F90" s="2" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
+      <c r="F90" s="2" t="inlineStr"/>
       <c r="G90" s="2" t="inlineStr">
         <is>
-          <t>Hissen uppfyller inte tillgänglighetskrav</t>
+          <t>Hyresgästen läggs ner i omorganisation</t>
         </is>
       </c>
       <c r="H90" s="2" t="inlineStr">
         <is>
-          <t>Hissen måste moderniseras för att klara nya myndighetskrav.</t>
+          <t>Moderbolaget stänger den lokala verksamheten och avtalet upphör.</t>
         </is>
       </c>
       <c r="I90" s="2" t="n">
@@ -4046,7 +4042,7 @@
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>KO-18</t>
+          <t>KO-17</t>
         </is>
       </c>
       <c r="C91" s="2" t="inlineStr">
@@ -4066,17 +4062,17 @@
       </c>
       <c r="F91" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G91" s="2" t="inlineStr">
         <is>
-          <t>Parkeringsdäcket har armeringsskador</t>
+          <t>Hissen uppfyller inte tillgänglighetskrav</t>
         </is>
       </c>
       <c r="H91" s="2" t="inlineStr">
         <is>
-          <t>Betongdäcket i garaget visar korrosion och måste renoveras.</t>
+          <t>Hissen måste moderniseras för att klara nya myndighetskrav.</t>
         </is>
       </c>
       <c r="I91" s="2" t="n">
@@ -4089,7 +4085,7 @@
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>KO-19</t>
+          <t>KO-18</t>
         </is>
       </c>
       <c r="C92" s="2" t="inlineStr">
@@ -4099,7 +4095,7 @@
       </c>
       <c r="D92" s="2" t="inlineStr">
         <is>
-          <t>villkorskort</t>
+          <t>underhallsvarning</t>
         </is>
       </c>
       <c r="E92" s="2" t="inlineStr">
@@ -4107,15 +4103,19 @@
           <t>ja</t>
         </is>
       </c>
-      <c r="F92" s="2" t="inlineStr"/>
+      <c r="F92" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
       <c r="G92" s="2" t="inlineStr">
         <is>
-          <t>Fastighetsskatten justeras för äldre bestånd</t>
+          <t>Parkeringsdäcket har armeringsskador</t>
         </is>
       </c>
       <c r="H92" s="2" t="inlineStr">
         <is>
-          <t>Villkor: fastigheter i energiklass D eller sämre får −1 DN.</t>
+          <t>Betongdäcket i garaget visar korrosion och måste renoveras.</t>
         </is>
       </c>
       <c r="I92" s="2" t="n">
@@ -4128,7 +4128,7 @@
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t>KO-20</t>
+          <t>KO-19</t>
         </is>
       </c>
       <c r="C93" s="2" t="inlineStr">
@@ -4149,12 +4149,12 @@
       <c r="F93" s="2" t="inlineStr"/>
       <c r="G93" s="2" t="inlineStr">
         <is>
-          <t>Kreditgivaren granskar portföljens miljöprofil</t>
+          <t>Fastighetsskatten justeras för äldre bestånd</t>
         </is>
       </c>
       <c r="H93" s="2" t="inlineStr">
         <is>
-          <t>Villkor: äger du 3 eller fler kontor — −1 DN på alla.</t>
+          <t>Villkor: fastigheter i energiklass D eller sämre får −1 DN.</t>
         </is>
       </c>
       <c r="I93" s="2" t="n">
@@ -4167,7 +4167,7 @@
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>KO-21</t>
+          <t>KO-20</t>
         </is>
       </c>
       <c r="C94" s="2" t="inlineStr">
@@ -4188,12 +4188,12 @@
       <c r="F94" s="2" t="inlineStr"/>
       <c r="G94" s="2" t="inlineStr">
         <is>
-          <t>Konjunkturen viker för kontorsmarknaden</t>
+          <t>Kreditgivaren granskar portföljens miljöprofil</t>
         </is>
       </c>
       <c r="H94" s="2" t="inlineStr">
         <is>
-          <t>Villkor: har fastigheten en vakant yta sedan tidigare — ytterligare −1 DN.</t>
+          <t>Villkor: äger du 3 eller fler kontor — −1 DN på alla.</t>
         </is>
       </c>
       <c r="I94" s="2" t="n">
@@ -4206,7 +4206,7 @@
       </c>
       <c r="B95" s="2" t="inlineStr">
         <is>
-          <t>KO-22</t>
+          <t>KO-21</t>
         </is>
       </c>
       <c r="C95" s="2" t="inlineStr">
@@ -4216,7 +4216,7 @@
       </c>
       <c r="D95" s="2" t="inlineStr">
         <is>
-          <t>engangskassa_plus</t>
+          <t>villkorskort</t>
         </is>
       </c>
       <c r="E95" s="2" t="inlineStr">
@@ -4224,19 +4224,15 @@
           <t>ja</t>
         </is>
       </c>
-      <c r="F95" s="2" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
+      <c r="F95" s="2" t="inlineStr"/>
       <c r="G95" s="2" t="inlineStr">
         <is>
-          <t>Avflyttande hyresgäst löser ut kontraktet</t>
+          <t>Konjunkturen viker för kontorsmarknaden</t>
         </is>
       </c>
       <c r="H95" s="2" t="inlineStr">
         <is>
-          <t>Företaget betalar avgångsvederlag för att lämna i förtid.</t>
+          <t>Villkor: har fastigheten en vakant yta sedan tidigare — ytterligare −1 DN.</t>
         </is>
       </c>
       <c r="I95" s="2" t="n">
@@ -4249,7 +4245,7 @@
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>KO-23</t>
+          <t>KO-22</t>
         </is>
       </c>
       <c r="C96" s="2" t="inlineStr">
@@ -4259,7 +4255,7 @@
       </c>
       <c r="D96" s="2" t="inlineStr">
         <is>
-          <t>engangskassa_minus</t>
+          <t>engangskassa_plus</t>
         </is>
       </c>
       <c r="E96" s="2" t="inlineStr">
@@ -4269,17 +4265,17 @@
       </c>
       <c r="F96" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="G96" s="2" t="inlineStr">
         <is>
-          <t>Elcentralen måste uppgraderas akut</t>
+          <t>Avflyttande hyresgäst löser ut kontraktet</t>
         </is>
       </c>
       <c r="H96" s="2" t="inlineStr">
         <is>
-          <t>Ökad effektbehov hos hyresgästerna kräver omedelbar förstärkning.</t>
+          <t>Företaget betalar avgångsvederlag för att lämna i förtid.</t>
         </is>
       </c>
       <c r="I96" s="2" t="n">
@@ -4292,7 +4288,7 @@
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>KO-24</t>
+          <t>KO-23</t>
         </is>
       </c>
       <c r="C97" s="2" t="inlineStr">
@@ -4312,17 +4308,17 @@
       </c>
       <c r="F97" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G97" s="2" t="inlineStr">
         <is>
-          <t>Sprinklerhuvud löser ut felaktigt</t>
+          <t>Elcentralen måste uppgraderas akut</t>
         </is>
       </c>
       <c r="H97" s="2" t="inlineStr">
         <is>
-          <t>Vattenskadan efter felutlösningen måste åtgärdas omgående.</t>
+          <t>Ökad effektbehov hos hyresgästerna kräver omedelbar förstärkning.</t>
         </is>
       </c>
       <c r="I97" s="2" t="n">
@@ -4335,7 +4331,7 @@
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>KO-25</t>
+          <t>KO-24</t>
         </is>
       </c>
       <c r="C98" s="2" t="inlineStr">
@@ -4345,7 +4341,7 @@
       </c>
       <c r="D98" s="2" t="inlineStr">
         <is>
-          <t>forkop</t>
+          <t>engangskassa_minus</t>
         </is>
       </c>
       <c r="E98" s="2" t="inlineStr">
@@ -4353,15 +4349,19 @@
           <t>ja</t>
         </is>
       </c>
-      <c r="F98" s="2" t="inlineStr"/>
+      <c r="F98" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
       <c r="G98" s="2" t="inlineStr">
         <is>
-          <t>Tips om kontorsfastighet i city</t>
+          <t>Sprinklerhuvud löser ut felaktigt</t>
         </is>
       </c>
       <c r="H98" s="2" t="inlineStr">
         <is>
-          <t>Behåll på hand. Ger förstaval när ett kontor sätts till budgivning.</t>
+          <t>Vattenskadan efter felutlösningen måste åtgärdas omgående.</t>
         </is>
       </c>
       <c r="I98" s="2" t="n">
@@ -4374,7 +4374,7 @@
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
-          <t>KO-26</t>
+          <t>KO-25</t>
         </is>
       </c>
       <c r="C99" s="2" t="inlineStr">
@@ -4395,12 +4395,12 @@
       <c r="F99" s="2" t="inlineStr"/>
       <c r="G99" s="2" t="inlineStr">
         <is>
-          <t>Kontakt hos kommersiell fastighetsmäklare</t>
+          <t>Tips om kontorsfastighet i city</t>
         </is>
       </c>
       <c r="H99" s="2" t="inlineStr">
         <is>
-          <t>Behåll på hand. Kortet ger dig förstaval nästa gång ett kontor går till budgivning.</t>
+          <t>Behåll på hand. Ger förstaval när ett kontor sätts till budgivning.</t>
         </is>
       </c>
       <c r="I99" s="2" t="n">
@@ -4413,17 +4413,17 @@
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>HR-24</t>
+          <t>KO-26</t>
         </is>
       </c>
       <c r="C100" s="2" t="inlineStr">
         <is>
-          <t>HYRESRÄTT</t>
+          <t>KONTOR</t>
         </is>
       </c>
       <c r="D100" s="2" t="inlineStr">
         <is>
-          <t>utveckling</t>
+          <t>forkop</t>
         </is>
       </c>
       <c r="E100" s="2" t="inlineStr">
@@ -4434,12 +4434,12 @@
       <c r="F100" s="2" t="inlineStr"/>
       <c r="G100" s="2" t="inlineStr">
         <is>
-          <t>Lyckad hyresförhandling</t>
+          <t>Kontakt hos kommersiell fastighetsmäklare</t>
         </is>
       </c>
       <c r="H100" s="2" t="inlineStr">
         <is>
-          <t>Förhandlingen med hyresgästföreningen går smidigt och ger erfarenhet. Lägg en utvecklingsbricka på din FC om den har fastighetens typ, annars på din FS.</t>
+          <t>Behåll på hand. Kortet ger dig förstaval nästa gång ett kontor går till budgivning.</t>
         </is>
       </c>
       <c r="I100" s="2" t="n">
@@ -4569,12 +4569,12 @@
       </c>
       <c r="B104" s="2" t="inlineStr">
         <is>
-          <t>HR-25</t>
+          <t>FO-25</t>
         </is>
       </c>
       <c r="C104" s="2" t="inlineStr">
         <is>
-          <t>HYRESRÄTT</t>
+          <t>FÖRSKOLA</t>
         </is>
       </c>
       <c r="D104" s="2" t="inlineStr">
@@ -4590,12 +4590,12 @@
       <c r="F104" s="2" t="inlineStr"/>
       <c r="G104" s="2" t="inlineStr">
         <is>
-          <t>Skadefritt år belönas</t>
+          <t>Kommunen förlänger avtalet i god tid</t>
         </is>
       </c>
       <c r="H104" s="2" t="inlineStr">
         <is>
-          <t>Försäkringsbolaget sänker självrisken efter ett år utan skador. Ta en riskbuffert.</t>
+          <t>Hyresgästen visar att den vill stanna länge. Ta en riskbuffert.</t>
         </is>
       </c>
       <c r="I104" s="2" t="n">
@@ -4608,12 +4608,12 @@
       </c>
       <c r="B105" s="2" t="inlineStr">
         <is>
-          <t>FO-25</t>
+          <t>LO-28</t>
         </is>
       </c>
       <c r="C105" s="2" t="inlineStr">
         <is>
-          <t>FÖRSKOLA</t>
+          <t>LOKAL</t>
         </is>
       </c>
       <c r="D105" s="2" t="inlineStr">
@@ -4629,12 +4629,12 @@
       <c r="F105" s="2" t="inlineStr"/>
       <c r="G105" s="2" t="inlineStr">
         <is>
-          <t>Kommunen förlänger avtalet i god tid</t>
+          <t>Hyresgästen ställer extra säkerhet</t>
         </is>
       </c>
       <c r="H105" s="2" t="inlineStr">
         <is>
-          <t>Hyresgästen visar att den vill stanna länge. Ta en riskbuffert.</t>
+          <t>Den nya hyresgästen lämnar en bankgaranti utöver det vanliga. Ta en riskbuffert.</t>
         </is>
       </c>
       <c r="I105" s="2" t="n">
@@ -4647,12 +4647,12 @@
       </c>
       <c r="B106" s="2" t="inlineStr">
         <is>
-          <t>LO-28</t>
+          <t>KO-28</t>
         </is>
       </c>
       <c r="C106" s="2" t="inlineStr">
         <is>
-          <t>LOKAL</t>
+          <t>KONTOR</t>
         </is>
       </c>
       <c r="D106" s="2" t="inlineStr">
@@ -4668,54 +4668,15 @@
       <c r="F106" s="2" t="inlineStr"/>
       <c r="G106" s="2" t="inlineStr">
         <is>
-          <t>Hyresgästen ställer extra säkerhet</t>
+          <t>Långt hyresavtal med stark hyresgäst</t>
         </is>
       </c>
       <c r="H106" s="2" t="inlineStr">
         <is>
-          <t>Den nya hyresgästen lämnar en bankgaranti utöver det vanliga. Ta en riskbuffert.</t>
+          <t>Ett börsbolag skriver på för tio år. Ta en riskbuffert.</t>
         </is>
       </c>
       <c r="I106" s="2" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="107">
-      <c r="A107" s="2" t="n">
-        <v>106</v>
-      </c>
-      <c r="B107" s="2" t="inlineStr">
-        <is>
-          <t>KO-28</t>
-        </is>
-      </c>
-      <c r="C107" s="2" t="inlineStr">
-        <is>
-          <t>KONTOR</t>
-        </is>
-      </c>
-      <c r="D107" s="2" t="inlineStr">
-        <is>
-          <t>riskbuffert</t>
-        </is>
-      </c>
-      <c r="E107" s="2" t="inlineStr">
-        <is>
-          <t>ja</t>
-        </is>
-      </c>
-      <c r="F107" s="2" t="inlineStr"/>
-      <c r="G107" s="2" t="inlineStr">
-        <is>
-          <t>Långt hyresavtal med stark hyresgäst</t>
-        </is>
-      </c>
-      <c r="H107" s="2" t="inlineStr">
-        <is>
-          <t>Ett börsbolag skriver på för tio år. Ta en riskbuffert.</t>
-        </is>
-      </c>
-      <c r="I107" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -4766,7 +4727,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C107"/>
+  <dimension ref="A1:C106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4842,7 +4803,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Skötsamma hyresgäster stannar</t>
+          <t>Lägenhet står tom</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -4857,7 +4818,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Garageplatser fulltecknade</t>
+          <t>Andrahandsuthyrning upptäcks</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -4872,7 +4833,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Tvättstugebokningar ökar</t>
+          <t>Nya termostatventiler monteras</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -4887,7 +4848,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Lägenhet står tom</t>
+          <t>Fjärrvärmeväxlare åldras</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -4902,7 +4863,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Andrahandsuthyrning upptäcks</t>
+          <t>Stammar i akut behov av byte</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -4917,7 +4878,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Källarförråd vattenskadat</t>
+          <t>Taket läcker vid slagregn</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -4932,7 +4893,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Nya termostatventiler monteras</t>
+          <t>Hissen klarar inte besiktning</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -4947,7 +4908,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Tätning av fönster lyckas</t>
+          <t>Boverket skärper energikrav</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -4962,7 +4923,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Fjärrvärmeväxlare åldras</t>
+          <t>Portföljen granskas av försäkringsbolag</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -4977,7 +4938,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Kommunen tecknar blockhyra</t>
+          <t>Retroaktiv hyra betalas ut</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -4992,7 +4953,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Stammar i akut behov av byte</t>
+          <t>Försäkringsersättning för stormskada</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -5007,7 +4968,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Taket läcker vid slagregn</t>
+          <t>Akut sanering av mögel</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -5022,7 +4983,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Hissen klarar inte besiktning</t>
+          <t>Tips om hyresfastighet i grannkvarteret</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -5037,7 +4998,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Boverket skärper energikrav</t>
+          <t>Mäklarkontakt i bostadsbolaget</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -5052,7 +5013,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Portföljen granskas av försäkringsbolag</t>
+          <t>Lyckad hyresförhandling</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -5067,7 +5028,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Retroaktiv hyra betalas ut</t>
+          <t>Skadefritt år belönas</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -5082,7 +5043,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Försäkringsersättning för stormskada</t>
+          <t>Lugnt kvartal i huset</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -5097,7 +5058,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Akut sanering av mögel</t>
+          <t>Hyresavierna går ut som vanligt</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -5112,7 +5073,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Tips om hyresfastighet i grannkvarteret</t>
+          <t>Ordinarie fastighetsskötsel</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -5127,7 +5088,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Mäklarkontakt i bostadsbolaget</t>
+          <t>Årets hyresförhandling klar</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -5142,7 +5103,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Kommunen förlänger avtalet</t>
+          <t>Stabilt boende</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -5157,7 +5118,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Fler avdelningar öppnas</t>
+          <t>Kommunen förlänger avtalet</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -5172,7 +5133,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Indexklausul ger högre hyra</t>
+          <t>Fler avdelningar öppnas</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -5187,7 +5148,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Föräldrakooperativ flyttar in</t>
+          <t>Indexklausul ger högre hyra</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -5202,7 +5163,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Gården nyttjas av flera verksamheter</t>
+          <t>Föräldrakooperativ flyttar in</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -5217,7 +5178,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Köket hyrs ut för catering</t>
+          <t>Gården nyttjas av flera verksamheter</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -5232,7 +5193,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Avdelning läggs vilande</t>
+          <t>Köket hyrs ut för catering</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -5247,7 +5208,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Personalutrymme underutnyttjat</t>
+          <t>Avdelning läggs vilande</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -5262,7 +5223,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Fuktskada i grovkök</t>
+          <t>Personalutrymme underutnyttjat</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -5277,7 +5238,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Solavskärmning minskar kylbehov</t>
+          <t>Fuktskada i grovkök</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -5292,7 +5253,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Behovsstyrd ventilation installeras</t>
+          <t>Solavskärmning minskar kylbehov</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -5307,7 +5268,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Undercentralen är original</t>
+          <t>Behovsstyrd ventilation installeras</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -5322,7 +5283,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Kommunen bygger ut avtalet till hela huset</t>
+          <t>Undercentralen är original</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -5337,7 +5298,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Lekutrustningen underkänns</t>
+          <t>Kommunen bygger ut avtalet till hela huset</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -5352,7 +5313,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Ventilationen klarar inte OVK</t>
+          <t>Lekutrustningen underkänns</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -5367,7 +5328,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Fasaden har frostsprängts</t>
+          <t>Ventilationen klarar inte OVK</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -5382,7 +5343,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Kommunen inför skärpta miljökrav</t>
+          <t>Fasaden har frostsprängts</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -5397,7 +5358,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Skolinspektionen granskar fastighetsbeståndet</t>
+          <t>Kommunen inför skärpta miljökrav</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -5412,7 +5373,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Kommunalt underhållsbidrag betalas ut</t>
+          <t>Skolinspektionen granskar fastighetsbeståndet</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -5427,7 +5388,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Försäkringsersättning för skadegörelse</t>
+          <t>Kommunalt underhållsbidrag betalas ut</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -5442,7 +5403,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Statligt investeringsstöd för förskolor</t>
+          <t>Försäkringsersättning för skadegörelse</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -5457,7 +5418,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Tips om förskola på kommunens lista</t>
+          <t>Statligt investeringsstöd för förskolor</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -5472,7 +5433,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Kontakt på kommunens fastighetskontor</t>
+          <t>Tips om förskola på kommunens lista</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -5487,7 +5448,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Omsättningshyra slår väl ut</t>
+          <t>Kontakt på kommunens fastighetskontor</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -5502,7 +5463,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Ny hyresgäst tecknar långt kontrakt</t>
+          <t>Omsättningshyra slår väl ut</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -5517,7 +5478,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Skyltläget lockar ny verksamhet</t>
+          <t>Ny hyresgäst tecknar långt kontrakt</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -5532,7 +5493,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Restaurangen bygger ut uteserveringen</t>
+          <t>Skyltläget lockar ny verksamhet</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -5547,7 +5508,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Popup-butik hyr in sig kort</t>
+          <t>Restaurangen bygger ut uteserveringen</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -5562,7 +5523,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Butiken sänker sin omsättning</t>
+          <t>Popup-butik hyr in sig kort</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -5577,7 +5538,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Lokal svår att hyra ut vidare</t>
+          <t>Butiken sänker sin omsättning</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -5592,7 +5553,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Konkurrerande handelsplats öppnar</t>
+          <t>Lokal svår att hyra ut vidare</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -5607,7 +5568,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Fettavskiljaren läcker smått</t>
+          <t>Konkurrerande handelsplats öppnar</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -5622,7 +5583,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Skyltfönster krossat en tid</t>
+          <t>Fettavskiljaren läcker smått</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -5637,7 +5598,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Hyresrabatt förhandlas fram i det tysta</t>
+          <t>Skyltfönster krossat en tid</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -5652,7 +5613,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Ny LED-belysning i butiksytan</t>
+          <t>Hyresrabatt förhandlas fram i det tysta</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -5667,7 +5628,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Kylanläggningen börjar dra mer el</t>
+          <t>Ny LED-belysning i butiksytan</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -5682,7 +5643,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Ventilationsaggregatet är original</t>
+          <t>Kylanläggningen börjar dra mer el</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -5697,7 +5658,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Ankarhyresgäst tecknar tioårsavtal</t>
+          <t>Ventilationsaggregatet är original</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -5712,7 +5673,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Ankarhyresgästen går i konkurs</t>
+          <t>Ankarhyresgäst tecknar tioårsavtal</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -5727,7 +5688,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Golvet i handelslokalen är utslitet</t>
+          <t>Ankarhyresgästen går i konkurs</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -5742,7 +5703,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Fasaden mot gatan vittrar</t>
+          <t>Golvet i handelslokalen är utslitet</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -5757,7 +5718,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>E-handeln tar ytterligare mark</t>
+          <t>Fasaden mot gatan vittrar</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -5772,7 +5733,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Kommunen skärper energikrav för handel</t>
+          <t>E-handeln tar ytterligare mark</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -5787,7 +5748,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Avflyttande hyresgäst betalar avgångsvederlag</t>
+          <t>Kommunen skärper energikrav för handel</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -5802,7 +5763,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Försäkringsersättning efter vattenskada</t>
+          <t>Avflyttande hyresgäst betalar avgångsvederlag</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -5817,7 +5778,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Akutsanering av fettavskiljare</t>
+          <t>Försäkringsersättning efter vattenskada</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -5832,7 +5793,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Klotter saneras akut på fasaden</t>
+          <t>Akutsanering av fettavskiljare</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -5847,7 +5808,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Tips om butikslokal i köpstark gata</t>
+          <t>Klotter saneras akut på fasaden</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -5862,7 +5823,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Kontakt hos fastighetsmäklare i city</t>
+          <t>Tips om butikslokal i köpstark gata</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -5877,7 +5838,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Hyresgästen expanderar på plats</t>
+          <t>Kontakt hos fastighetsmäklare i city</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -5892,7 +5853,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Långt avtal förlängs i förtid</t>
+          <t>Hyresgästen expanderar på plats</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -5907,7 +5868,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Kontorshotell fyller vakanta ytor</t>
+          <t>Långt avtal förlängs i förtid</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -5922,7 +5883,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Indexuppräkning ger högre hyra</t>
+          <t>Kontorshotell fyller vakanta ytor</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -5937,7 +5898,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Del av våningsplan står tomt</t>
+          <t>Indexuppräkning ger högre hyra</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -5952,7 +5913,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Distansarbete minskar ytbehovet</t>
+          <t>Del av våningsplan står tomt</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -5967,7 +5928,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Konferensrum står obokat</t>
+          <t>Distansarbete minskar ytbehovet</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -5982,7 +5943,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Elkapaciteten börjar bli en flaskhals</t>
+          <t>Konferensrum står obokat</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -5997,7 +5958,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Reception underutnyttjad</t>
+          <t>Elkapaciteten börjar bli en flaskhals</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -6012,7 +5973,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Parkeringsgaraget har lediga platser</t>
+          <t>Reception underutnyttjad</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
@@ -6027,7 +5988,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Behovsstyrd belysning installeras</t>
+          <t>Parkeringsgaraget har lediga platser</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
@@ -6042,7 +6003,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Kylmaskinen för komfortkyla åldras</t>
+          <t>Behovsstyrd belysning installeras</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -6057,7 +6018,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Klimatskalet läcker värme</t>
+          <t>Kylmaskinen för komfortkyla åldras</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
@@ -6072,7 +6033,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Storbolag flyttar in på tioårsavtal</t>
+          <t>Klimatskalet läcker värme</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
@@ -6087,7 +6048,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Storhyresgästen flyttar till nybygge</t>
+          <t>Storbolag flyttar in på tioårsavtal</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
@@ -6102,7 +6063,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Hyresgästen läggs ner i omorganisation</t>
+          <t>Storhyresgästen flyttar till nybygge</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
@@ -6117,7 +6078,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Hissen uppfyller inte tillgänglighetskrav</t>
+          <t>Hyresgästen läggs ner i omorganisation</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
@@ -6132,7 +6093,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Parkeringsdäcket har armeringsskador</t>
+          <t>Hissen uppfyller inte tillgänglighetskrav</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
@@ -6147,7 +6108,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Fastighetsskatten justeras för äldre bestånd</t>
+          <t>Parkeringsdäcket har armeringsskador</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
@@ -6162,7 +6123,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Kreditgivaren granskar portföljens miljöprofil</t>
+          <t>Fastighetsskatten justeras för äldre bestånd</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
@@ -6177,7 +6138,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Konjunkturen viker för kontorsmarknaden</t>
+          <t>Kreditgivaren granskar portföljens miljöprofil</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
@@ -6192,7 +6153,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Avflyttande hyresgäst löser ut kontraktet</t>
+          <t>Konjunkturen viker för kontorsmarknaden</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
@@ -6207,7 +6168,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Elcentralen måste uppgraderas akut</t>
+          <t>Avflyttande hyresgäst löser ut kontraktet</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
@@ -6222,7 +6183,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Sprinklerhuvud löser ut felaktigt</t>
+          <t>Elcentralen måste uppgraderas akut</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
@@ -6237,7 +6198,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Tips om kontorsfastighet i city</t>
+          <t>Sprinklerhuvud löser ut felaktigt</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
@@ -6252,7 +6213,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Kontakt hos kommersiell fastighetsmäklare</t>
+          <t>Tips om kontorsfastighet i city</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
@@ -6267,7 +6228,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Lyckad hyresförhandling</t>
+          <t>Kontakt hos kommersiell fastighetsmäklare</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
@@ -6327,7 +6288,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>Skadefritt år belönas</t>
+          <t>Kommunen förlänger avtalet i god tid</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
@@ -6342,7 +6303,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>Kommunen förlänger avtalet i god tid</t>
+          <t>Hyresgästen ställer extra säkerhet</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
@@ -6357,25 +6318,10 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>Hyresgästen ställer extra säkerhet</t>
+          <t>Långt hyresavtal med stark hyresgäst</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
-        <is>
-          <t>ej bestämt</t>
-        </is>
-      </c>
-    </row>
-    <row r="107">
-      <c r="A107" t="n">
-        <v>106</v>
-      </c>
-      <c r="B107" t="inlineStr">
-        <is>
-          <t>Långt hyresavtal med stark hyresgäst</t>
-        </is>
-      </c>
-      <c r="C107" t="inlineStr">
         <is>
           <t>ej bestämt</t>
         </is>
@@ -6671,7 +6617,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>106 (kortspecen: 106)</t>
+          <t>105 (kortspecen: 105)</t>
         </is>
       </c>
     </row>

</xml_diff>